<commit_message>
Fix OI-77 SA-review: 5 follow-up issues from senior architect
- capture_pipeline_run.py: remove duplicate detected_domain key (bug)
- refresh_golden_step6.py: remove dead detected_domain assignment
- app.py: fix x-or-x tautology in replay detected_domain read
- test_classification.py: add two behavioral assertions to
  test_domain_extractability_contract (gate expression + non-empty domains)
- Spec/haystacked_platform_config.xlsx: delete is_agv_amr row from
  Basic Extraction Schema tab (source fix — prevents re-entry on
  next generate_all.py run). 247 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_platform_config.xlsx
+++ b/Spec/haystacked_platform_config.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -823,39 +823,39 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>is_agv_amr</t>
+          <t>summary</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>true if document requests AGV, AMR, automated intralogistics vehicles, VNA robots, or self-driving warehouse/factory transport. true if words AGV, AMR, or VNA appear.</t>
+          <t>1-2 sentence summary of what is being procured and who the buyer is.</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>missing_info</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>array</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -865,37 +865,10 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>1-2 sentence summary of what is being procured and who the buyer is.</t>
+          <t>List of important fields that cannot be determined from the document (e.g. ["lifting_height_mm", "aisle_width_mm"]).</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>missing_info</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>List of important fields that cannot be determined from the document (e.g. ["lifting_height_mm", "aisle_width_mm"]).</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>